<commit_message>
Make inventory spreadsheet paths relative to the repo root
</commit_message>
<xml_diff>
--- a/notebook_data_obj_inventory.xlsx
+++ b/notebook_data_obj_inventory.xlsx
@@ -927,7 +927,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_linear/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_linear/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -955,7 +955,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_quadratic/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_quadratic/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_exp/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_exp/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_const/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_const/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_quadratic/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_quadratic/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F9" s="15" t="n">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_exp/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_exp/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F10" s="15" t="n">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_linear/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_linear/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F11" s="15" t="n">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_11/dataX2num_11/dataTnum_9/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_linear/dataGamma_1/dataNoisePercent_5/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_11/dataX2num_11/dataTnum_9/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_linear/dataGamma_1/dataNoisePercent_5/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_1/dataNoisePercent_1/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_1/dataNoisePercent_1/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_linear/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_linear/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_1/dataNoisePercent_1/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_1/dataNoisePercent_1/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>/Users/willa954/Desktop/Git-personal/Hyperparam/hyperparam-selection/Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
+          <t>Training/data/dataObj/dataX1num_38/dataX2num_1/dataTnum_5/dataK_1/dataICLabel_cos/dataDiffLabel_const/dataGrowLabel_zero/dataGamma_0/dataNoisePercent_0/dataNoiseSeed_0/data_obj.npy</t>
         </is>
       </c>
       <c r="F8" s="15" t="n">

</xml_diff>